<commit_message>
Team project sync’ed with translations and QE data
</commit_message>
<xml_diff>
--- a/exports/test_en--ar_OMT_QE_scores.xlsx
+++ b/exports/test_en--ar_OMT_QE_scores.xlsx
@@ -425,100 +425,262 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>src</t>
+          <t>file</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source_text</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>target_text</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>repetition</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ice_match</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>in_scope</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>mt</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>score</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>qe_score</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>file_with_formatting.docx</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NFDBB2FA9-tu1_0</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>This is a &lt;g1&gt;bolded&lt;/g1&gt; word.</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>هذه كلمة &lt;g1&gt;جريئة&lt;/g1&gt;.</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>0.5071799755096436</v>
-      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>هذه كلمة بخط &lt;g1&gt;عريض&lt;/g1&gt;.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>file_with_formatting.docx</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NFDBB2FA9-tu2_0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>This is my best sentence yet.</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>هذه أفضل جملة لي حتى الآن.</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>0.8854201436042786</v>
-      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>هذه أفضل جملة لي حتى الآن.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>foo.xml</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1_0</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>This is a repeated sentence.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>هذه جملة مكررة.</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>0.910571277141571</v>
-      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FIRST</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>هذه جملة مكررة.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>foo.xml</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2_0</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>The following is addressed to a girl:</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>يتم توجيه ما يلي إلى فتاة:</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>0.8859434723854065</v>
-      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FIRST</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ما يلي موجه إلى فتاة:</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>foo.xml</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3_0</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>What is your age?</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>كم عمرك ؟</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>0.9172203540802002</v>
-      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FIRST</t>
+        </is>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>كم عمرك؟</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>